<commit_message>
Tighten graph topological-order review details
</commit_message>
<xml_diff>
--- a/task-reviews/graph/task_graph_order_topological_position/task_graph_order_topological_position.xlsx
+++ b/task-reviews/graph/task_graph_order_topological_position/task_graph_order_topological_position.xlsx
@@ -1778,7 +1778,7 @@
 Evidence rule: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer rule: set "answer" to the 1-based position of node C in that order as an integer.
 Example JSON:
-{"evidence":["B","D","H","J"],"answer":3}</t>
+{"evidence":["A","B","C","D","E"],"answer":3}</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1842,7 +1842,7 @@
 Evidence rule: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer rule: set "answer" to the 1-based position of node B in that order as an integer.
 Example JSON:
-{"evidence":["B","D","H","J"],"answer":3}</t>
+{"evidence":["A","B","C","D","E"],"answer":3}</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1906,7 +1906,7 @@
 Evidence requirement: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer format: set "answer" to the 1-based position of node F in that order as an integer.
 Example JSON:
-{"evidence":["B","D","H","J"],"answer":3}</t>
+{"evidence":["A","B","C","D","E"],"answer":3}</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1970,7 +1970,7 @@
 Evidence requirement: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer format: set "answer" to the 1-based position of node 1 in that order as an integer.
 Example JSON:
-{"evidence":["2","5","8","9"],"answer":3}</t>
+{"evidence":["1","2","3","4","5"],"answer":3}</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -2034,7 +2034,7 @@
 Evidence requirement: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer format: set "answer" to the 1-based position of node D in that order as an integer.
 Example JSON:
-{"evidence":["B","D","H","J"],"answer":3}</t>
+{"evidence":["A","B","C","D","E"],"answer":3}</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2098,7 +2098,7 @@
 Evidence requirement: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer format: set "answer" to the 1-based position of node G in that order as an integer.
 Example JSON:
-{"evidence":["B","D","H","J"],"answer":3}</t>
+{"evidence":["A","B","C","D","E"],"answer":3}</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -2162,7 +2162,7 @@
 Evidence requirement: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer format: set "answer" to the 1-based position of node 5 in that order as an integer.
 Example JSON:
-{"evidence":["2","5","8","9"],"answer":3}</t>
+{"evidence":["1","2","3","4","5"],"answer":3}</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -2226,7 +2226,7 @@
 Evidence field: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer field: set "answer" to the 1-based position of node 3 in that order as an integer.
 Example JSON:
-{"evidence":["2","5","8","9"],"answer":3}</t>
+{"evidence":["1","2","3","4","5"],"answer":3}</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -2290,7 +2290,7 @@
 Evidence field: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer field: set "answer" to the 1-based position of node A in that order as an integer.
 Example JSON:
-{"evidence":["B","D","H","J"],"answer":3}</t>
+{"evidence":["A","B","C","D","E"],"answer":3}</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -2354,7 +2354,7 @@
 Evidence field: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer field: set "answer" to the 1-based position of node C in that order as an integer.
 Example JSON:
-{"evidence":["B","D","H","J"],"answer":3}</t>
+{"evidence":["A","B","C","D","E"],"answer":3}</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -2418,7 +2418,7 @@
 Evidence rule: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer rule: set "answer" to the 1-based position of node 1 in that order as an integer.
 Example JSON:
-{"evidence":["2","5","8","9"],"answer":3}</t>
+{"evidence":["1","2","3","4","5"],"answer":3}</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -2482,7 +2482,7 @@
 Evidence requirement: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer format: set "answer" to the 1-based position of node 6 in that order as an integer.
 Example JSON:
-{"evidence":["2","5","8","9"],"answer":3}</t>
+{"evidence":["1","2","3","4","5"],"answer":3}</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -2546,7 +2546,7 @@
 Evidence field: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer field: set "answer" to the 1-based position of node 2 in that order as an integer.
 Example JSON:
-{"evidence":["2","5","8","9"],"answer":3}</t>
+{"evidence":["1","2","3","4","5"],"answer":3}</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -2610,7 +2610,7 @@
 Evidence format: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer requirement: set "answer" to the 1-based position of node 3 in that order as an integer.
 Example JSON:
-{"evidence":["2","5","8","9"],"answer":3}</t>
+{"evidence":["1","2","3","4","5"],"answer":3}</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -2674,7 +2674,7 @@
 Evidence field: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer field: set "answer" to the 1-based position of node 2 in that order as an integer.
 Example JSON:
-{"evidence":["2","5","8","9"],"answer":3}</t>
+{"evidence":["1","2","3","4","5"],"answer":3}</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -2738,7 +2738,7 @@
 Evidence field: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer field: set "answer" to the 1-based position of node G in that order as an integer.
 Example JSON:
-{"evidence":["B","D","H","J"],"answer":3}</t>
+{"evidence":["A","B","C","D","E"],"answer":3}</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -2802,7 +2802,7 @@
 Evidence rule: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer rule: set "answer" to the 1-based position of node C in that order as an integer.
 Example JSON:
-{"evidence":["B","D","H","J"],"answer":3}</t>
+{"evidence":["A","B","C","D","E"],"answer":3}</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -2866,7 +2866,7 @@
 Evidence requirement: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer format: set "answer" to the 1-based position of node 6 in that order as an integer.
 Example JSON:
-{"evidence":["2","5","8","9"],"answer":3}</t>
+{"evidence":["1","2","3","4","5"],"answer":3}</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -2930,7 +2930,7 @@
 Evidence: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer: set "answer" to the 1-based position of node E in that order as an integer.
 Example JSON:
-{"evidence":["B","D","H","J"],"answer":3}</t>
+{"evidence":["A","B","C","D","E"],"answer":3}</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -2994,7 +2994,7 @@
 Evidence: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer: set "answer" to the 1-based position of node 1 in that order as an integer.
 Example JSON:
-{"evidence":["2","5","8","9"],"answer":3}</t>
+{"evidence":["1","2","3","4","5"],"answer":3}</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -3058,7 +3058,7 @@
 Evidence: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer: set "answer" to the 1-based position of node A in that order as an integer.
 Example JSON:
-{"evidence":["B","D","H","J"],"answer":3}</t>
+{"evidence":["A","B","C","D","E"],"answer":3}</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -3122,7 +3122,7 @@
 Evidence rule: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer rule: set "answer" to the 1-based position of node 1 in that order as an integer.
 Example JSON:
-{"evidence":["2","5","8","9"],"answer":3}</t>
+{"evidence":["1","2","3","4","5"],"answer":3}</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -3186,7 +3186,7 @@
 Evidence format: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer requirement: set "answer" to the 1-based position of node G in that order as an integer.
 Example JSON:
-{"evidence":["B","D","H","J"],"answer":3}</t>
+{"evidence":["A","B","C","D","E"],"answer":3}</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -3250,7 +3250,7 @@
 Evidence requirement: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer format: set "answer" to the 1-based position of node 4 in that order as an integer.
 Example JSON:
-{"evidence":["2","5","8","9"],"answer":3}</t>
+{"evidence":["1","2","3","4","5"],"answer":3}</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -3314,7 +3314,7 @@
 Evidence rule: set "evidence" to an ordered array containing all node labels in the unique topological order from first to last.
 Answer rule: set "answer" to the 1-based position of node C in that order as an integer.
 Example JSON:
-{"evidence":["B","D","H","J"],"answer":3}</t>
+{"evidence":["A","B","C","D","E"],"answer":3}</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">

</xml_diff>